<commit_message>
Data driven changes for the sign up process
</commit_message>
<xml_diff>
--- a/src/resources/testdata/TestData.xlsx
+++ b/src/resources/testdata/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PlaywrightPython\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KoyaRohitaBhavani\MyClarioPytestFramework\src\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44692B62-BA85-4092-9630-801F7519EABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF009A33-8073-4161-AEDB-24F63D6ADC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t>username</t>
   </si>
@@ -35,17 +35,68 @@
     <t>Steephen@1291</t>
   </si>
   <si>
-    <t>naveen.mandaji@bilvantis.io</t>
-  </si>
-  <si>
-    <t>Nikshith@1802</t>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>ConfirmPassword</t>
+  </si>
+  <si>
+    <t>TC_SIP_001</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Test@123</t>
+  </si>
+  <si>
+    <t>TC_SIP_002</t>
+  </si>
+  <si>
+    <t>Rohitha</t>
+  </si>
+  <si>
+    <t>Koya</t>
+  </si>
+  <si>
+    <t>TC_SIP_003</t>
+  </si>
+  <si>
+    <t>rohita.koya@bilvantis.io</t>
+  </si>
+  <si>
+    <t>Data4</t>
+  </si>
+  <si>
+    <t>testdata4@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -60,6 +111,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFC9D1D9"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,9 +148,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -391,6 +467,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.6328125" customWidth="1"/>
+    <col min="2" max="2" width="21.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -415,33 +495,127 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3E684D-AE02-477B-AD19-29320004CE66}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.453125" customWidth="1"/>
-    <col min="2" max="2" width="13.6328125" customWidth="1"/>
+    <col min="1" max="1" width="15.90625" customWidth="1"/>
+    <col min="2" max="2" width="22.6328125" customWidth="1"/>
+    <col min="3" max="3" width="36.81640625" customWidth="1"/>
+    <col min="4" max="4" width="30.08984375" customWidth="1"/>
+    <col min="5" max="5" width="20.7265625" customWidth="1"/>
+    <col min="6" max="6" width="20.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.90625" customWidth="1"/>
+    <col min="8" max="8" width="15.08984375" customWidth="1"/>
+    <col min="9" max="9" width="20.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3">
+        <v>9876543210</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3">
+        <v>9876543210</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="3">
+        <v>9876543210</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{36AF6B82-9DA4-42A8-893B-0AFB7E2DEB21}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{80F5AE94-2ADD-4C11-8484-86626CC8B76A}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{90D66AD6-0A0F-4215-B6A8-8FA7717EA794}"/>
+    <hyperlink ref="D4" r:id="rId2" display="mailto:rohita.koya@bilvantis.io" xr:uid="{55904C95-7E71-41DD-969F-F8713774F32E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>